<commit_message>
I3: improved modularity and working section
</commit_message>
<xml_diff>
--- a/capstone16_evals_n_metrics.xlsx
+++ b/capstone16_evals_n_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\problem_first_ai\capstore16_code\unblocking_icq_phase1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D24542A-DFC9-4742-BD48-D4A53ABB799F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{584FAB32-8B52-4017-9CCD-24FD09671241}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="860" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -713,7 +713,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -790,6 +790,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1672,11 +1673,11 @@
         <v>5</v>
       </c>
       <c r="G16" s="30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16" s="30">
         <f t="shared" si="0"/>
-        <v>3.3333333333333335</v>
+        <v>3.6666666666666665</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
@@ -1919,9 +1920,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8F20231-225F-46AD-A21B-6B0A933A566B}">
-  <dimension ref="A1"/>
+  <dimension ref="C3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="3" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C3" s="38"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
ppt by adding emailids and evals in template format
</commit_message>
<xml_diff>
--- a/capstone16_evals_n_metrics.xlsx
+++ b/capstone16_evals_n_metrics.xlsx
@@ -5,24 +5,25 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\problem_first_ai\capstore16_code\unblocking_icq_phase1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\backup_code\unblocking_icq_phase1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6950F88-26A8-47E0-95E2-611926515627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A310D4C-21A1-4A19-A390-74685B7538D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="896" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Iteration1_Evals" sheetId="10" r:id="rId1"/>
     <sheet name="Iteration2_Evals" sheetId="11" r:id="rId2"/>
-    <sheet name="other" sheetId="12" r:id="rId3"/>
-    <sheet name="1_LLM_Metrics" sheetId="2" r:id="rId4"/>
-    <sheet name="2_RAG_Metrics" sheetId="3" r:id="rId5"/>
-    <sheet name="3_SQL_Metrics" sheetId="4" r:id="rId6"/>
-    <sheet name="4_Application_Metrics" sheetId="5" r:id="rId7"/>
-    <sheet name="5_Cost_Metrics" sheetId="6" r:id="rId8"/>
-    <sheet name="6_User_Experience" sheetId="7" r:id="rId9"/>
-    <sheet name="8_Optimization_Impact" sheetId="9" r:id="rId10"/>
+    <sheet name="Iteration3_Evals" sheetId="13" r:id="rId3"/>
+    <sheet name="other" sheetId="12" r:id="rId4"/>
+    <sheet name="1_LLM_Metrics" sheetId="2" r:id="rId5"/>
+    <sheet name="2_RAG_Metrics" sheetId="3" r:id="rId6"/>
+    <sheet name="3_SQL_Metrics" sheetId="4" r:id="rId7"/>
+    <sheet name="4_Application_Metrics" sheetId="5" r:id="rId8"/>
+    <sheet name="5_Cost_Metrics" sheetId="6" r:id="rId9"/>
+    <sheet name="6_User_Experience" sheetId="7" r:id="rId10"/>
+    <sheet name="8_Optimization_Impact" sheetId="9" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1003" uniqueCount="432">
   <si>
     <t>Metric Name</t>
   </si>
@@ -1206,53 +1207,7 @@
     <t>Eval metrics/measurements</t>
   </si>
   <si>
-    <t>LLM API calls - Need rate limiting</t>
-  </si>
-  <si>
-    <t>prompt optimization (reduce token usage)</t>
-  </si>
-  <si>
-    <t>String limits to queries, uploaded documents etc</t>
-  </si>
-  <si>
-    <t>LLM 
-a)  output quality - json parsing 
-b) response relevance score
-c) Hallucination detection rate - citations.
-D) gap analysis completeness - 100%</t>
-  </si>
-  <si>
-    <t>Vector store queries - caching</t>
-  </si>
-  <si>
-    <t>RAG - query caching (redis/memory)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> LLM API token limit or requests limit</t>
-  </si>
-  <si>
-    <t>RAG
-relevance
-retrieval drift
-latency
-correctness</t>
-  </si>
-  <si>
-    <t>gap analysis -  RAG intensive &amp; long running
-- processing time
-- compute overhead</t>
-  </si>
-  <si>
-    <t>LLM response caching (in gap analysis) - hash-based</t>
-  </si>
-  <si>
-    <t>Monitor cost</t>
-  </si>
-  <si>
     <t>Database query optimization (by indexes)</t>
-  </si>
-  <si>
-    <t>Stale data</t>
   </si>
   <si>
     <t>RAG queries sequal execution in gap (asyncio)</t>
@@ -1426,14 +1381,80 @@
     <t>15 to 25 sec</t>
   </si>
   <si>
-    <t>Iteration #2 &amp; 3: Evals and measurements</t>
+    <t>Iteration #3: Evals and measurements</t>
+  </si>
+  <si>
+    <t>Iteration #2: Evals and measurements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LLM API calls </t>
+  </si>
+  <si>
+    <t>Iteration</t>
+  </si>
+  <si>
+    <t>prompt optimization</t>
+  </si>
+  <si>
+    <t>SQL metrics</t>
+  </si>
+  <si>
+    <t>LLM optimization</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> LLM API token limit or requests limit
+Better source coverage on RAG
+Top docs get more space (smart truncation)</t>
+  </si>
+  <si>
+    <t>computation time
+skip the validation every time if first retrive successful.: saves 2-3 seconds</t>
+  </si>
+  <si>
+    <t>RAG - 
+More focused answers</t>
+  </si>
+  <si>
+    <t>LLM prompts  &amp; RAG</t>
+  </si>
+  <si>
+    <t>Few shot
+LLM output</t>
+  </si>
+  <si>
+    <t>few shot
+Zero shot
+on prompts reduced data.</t>
+  </si>
+  <si>
+    <t>LLM token usage</t>
+  </si>
+  <si>
+    <t>LLM calls</t>
+  </si>
+  <si>
+    <t>avoid usage of Stale data</t>
+  </si>
+  <si>
+    <t>LLM Judge
+Hallucination</t>
+  </si>
+  <si>
+    <t>response time &lt; 30 sec
+Better diversity (MMR)
+Success rate.</t>
+  </si>
+  <si>
+    <t>relevance of answers on 
+Gap analysis.
+Completion of all the sections of the report.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1510,6 +1531,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1549,7 +1578,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -1783,11 +1812,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1816,10 +1882,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1846,29 +1908,38 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1897,7 +1968,24 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2213,36 +2301,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="32" t="s">
         <v>317</v>
       </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
     </row>
     <row r="2" spans="1:8" ht="36" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="13" t="s">
         <v>319</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="13" t="s">
         <v>320</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="14" t="s">
         <v>321</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="F2" s="14" t="s">
         <v>322</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="14" t="s">
         <v>323</v>
       </c>
-      <c r="H2" s="16" t="s">
+      <c r="H2" s="14" t="s">
         <v>324</v>
       </c>
     </row>
@@ -2250,379 +2338,379 @@
       <c r="A3" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="15" t="s">
         <v>326</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="16" t="s">
         <v>327</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="16" t="s">
         <v>328</v>
       </c>
-      <c r="E3" s="18">
-        <v>1</v>
-      </c>
-      <c r="F3" s="18">
-        <v>1</v>
-      </c>
-      <c r="G3" s="18">
-        <v>1</v>
-      </c>
-      <c r="H3" s="18">
+      <c r="E3" s="16">
+        <v>1</v>
+      </c>
+      <c r="F3" s="16">
+        <v>1</v>
+      </c>
+      <c r="G3" s="16">
+        <v>1</v>
+      </c>
+      <c r="H3" s="16">
         <f>AVERAGE(E3:G3)</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="15" t="s">
         <v>326</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="16" t="s">
         <v>330</v>
       </c>
-      <c r="E4" s="18">
-        <v>1</v>
-      </c>
-      <c r="F4" s="18">
-        <v>1</v>
-      </c>
-      <c r="G4" s="18">
-        <v>1</v>
-      </c>
-      <c r="H4" s="18">
+      <c r="E4" s="16">
+        <v>1</v>
+      </c>
+      <c r="F4" s="16">
+        <v>1</v>
+      </c>
+      <c r="G4" s="16">
+        <v>1</v>
+      </c>
+      <c r="H4" s="16">
         <f t="shared" ref="H4:H26" si="0">AVERAGE(E4:G4)</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="15" t="s">
         <v>326</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="16" t="s">
         <v>331</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="16" t="s">
         <v>332</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="16">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="16">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="G5" s="18">
+      <c r="G5" s="16">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="H5" s="18">
+      <c r="H5" s="16">
         <f t="shared" si="0"/>
         <v>5.3333333333333332E-3</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="15" t="s">
         <v>326</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="16" t="s">
         <v>333</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="16" t="s">
         <v>334</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="16">
         <v>0</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="16">
         <v>0.5</v>
       </c>
-      <c r="G6" s="18">
-        <v>1</v>
-      </c>
-      <c r="H6" s="18">
+      <c r="G6" s="16">
+        <v>1</v>
+      </c>
+      <c r="H6" s="16">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="15" t="s">
         <v>335</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="16" t="s">
         <v>336</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="16" t="s">
         <v>337</v>
       </c>
-      <c r="E7" s="18">
-        <v>1</v>
-      </c>
-      <c r="F7" s="18">
-        <v>1</v>
-      </c>
-      <c r="G7" s="18">
-        <v>1</v>
-      </c>
-      <c r="H7" s="18">
+      <c r="E7" s="16">
+        <v>1</v>
+      </c>
+      <c r="F7" s="16">
+        <v>1</v>
+      </c>
+      <c r="G7" s="16">
+        <v>1</v>
+      </c>
+      <c r="H7" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="15" t="s">
         <v>335</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="16" t="s">
         <v>338</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="16" t="s">
         <v>339</v>
       </c>
-      <c r="E8" s="18">
-        <v>1</v>
-      </c>
-      <c r="F8" s="18">
-        <v>1</v>
-      </c>
-      <c r="G8" s="18">
+      <c r="E8" s="16">
+        <v>1</v>
+      </c>
+      <c r="F8" s="16">
+        <v>1</v>
+      </c>
+      <c r="G8" s="16">
         <v>0.5</v>
       </c>
-      <c r="H8" s="18">
+      <c r="H8" s="16">
         <f t="shared" si="0"/>
         <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="15" t="s">
         <v>335</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="16" t="s">
         <v>340</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="16" t="s">
         <v>341</v>
       </c>
-      <c r="E9" s="18">
-        <v>1</v>
-      </c>
-      <c r="F9" s="18">
-        <v>1</v>
-      </c>
-      <c r="G9" s="18">
-        <v>1</v>
-      </c>
-      <c r="H9" s="18">
+      <c r="E9" s="16">
+        <v>1</v>
+      </c>
+      <c r="F9" s="16">
+        <v>1</v>
+      </c>
+      <c r="G9" s="16">
+        <v>1</v>
+      </c>
+      <c r="H9" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="15" t="s">
         <v>335</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="16" t="s">
         <v>342</v>
       </c>
-      <c r="E10" s="18">
-        <v>1</v>
-      </c>
-      <c r="F10" s="18">
-        <v>1</v>
-      </c>
-      <c r="G10" s="18">
-        <v>1</v>
-      </c>
-      <c r="H10" s="18">
+      <c r="E10" s="16">
+        <v>1</v>
+      </c>
+      <c r="F10" s="16">
+        <v>1</v>
+      </c>
+      <c r="G10" s="16">
+        <v>1</v>
+      </c>
+      <c r="H10" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="24" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="17" t="s">
         <v>343</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="18" t="s">
         <v>344</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="18" t="s">
         <v>345</v>
       </c>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20" t="e">
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="16" t="s">
         <v>347</v>
       </c>
-      <c r="E12" s="18">
-        <v>1</v>
-      </c>
-      <c r="F12" s="18">
-        <v>1</v>
-      </c>
-      <c r="G12" s="18">
-        <v>1</v>
-      </c>
-      <c r="H12" s="18">
+      <c r="E12" s="16">
+        <v>1</v>
+      </c>
+      <c r="F12" s="16">
+        <v>1</v>
+      </c>
+      <c r="G12" s="16">
+        <v>1</v>
+      </c>
+      <c r="H12" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="16" t="s">
         <v>348</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="16" t="s">
         <v>349</v>
       </c>
-      <c r="E13" s="18">
-        <v>1</v>
-      </c>
-      <c r="F13" s="18">
-        <v>1</v>
-      </c>
-      <c r="G13" s="18">
-        <v>1</v>
-      </c>
-      <c r="H13" s="18">
+      <c r="E13" s="16">
+        <v>1</v>
+      </c>
+      <c r="F13" s="16">
+        <v>1</v>
+      </c>
+      <c r="G13" s="16">
+        <v>1</v>
+      </c>
+      <c r="H13" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="16" t="s">
         <v>350</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="16" t="s">
         <v>351</v>
       </c>
-      <c r="E14" s="18">
-        <v>1</v>
-      </c>
-      <c r="F14" s="18">
-        <v>1</v>
-      </c>
-      <c r="G14" s="18">
-        <v>1</v>
-      </c>
-      <c r="H14" s="18">
+      <c r="E14" s="16">
+        <v>1</v>
+      </c>
+      <c r="F14" s="16">
+        <v>1</v>
+      </c>
+      <c r="G14" s="16">
+        <v>1</v>
+      </c>
+      <c r="H14" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="16" t="s">
         <v>352</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="16" t="s">
         <v>353</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="16">
         <v>5</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="16">
         <v>5</v>
       </c>
-      <c r="G15" s="18">
+      <c r="G15" s="16">
         <v>5</v>
       </c>
-      <c r="H15" s="18">
+      <c r="H15" s="16">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="16" t="s">
         <v>352</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="16" t="s">
         <v>354</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="16">
         <v>5</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="16">
         <v>5</v>
       </c>
-      <c r="G16" s="18">
-        <v>1</v>
-      </c>
-      <c r="H16" s="18">
+      <c r="G16" s="16">
+        <v>1</v>
+      </c>
+      <c r="H16" s="16">
         <f t="shared" si="0"/>
         <v>3.6666666666666665</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="16" t="s">
         <v>352</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="16" t="s">
         <v>355</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="16">
         <v>5</v>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="16">
         <v>5</v>
       </c>
-      <c r="G17" s="18">
+      <c r="G17" s="16">
         <v>5</v>
       </c>
-      <c r="H17" s="18">
+      <c r="H17" s="16">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="24" x14ac:dyDescent="0.35">
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="15" t="s">
         <v>356</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="16" t="s">
         <v>357</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="16" t="s">
         <v>358</v>
       </c>
-      <c r="E18" s="18">
+      <c r="E18" s="16">
         <v>9.0399999999999991</v>
       </c>
-      <c r="F18" s="18">
+      <c r="F18" s="16">
         <v>9.35</v>
       </c>
-      <c r="G18" s="18">
+      <c r="G18" s="16">
         <v>7.88</v>
       </c>
-      <c r="H18" s="18">
+      <c r="H18" s="16">
         <f t="shared" si="0"/>
         <v>8.7566666666666659</v>
       </c>
@@ -2631,43 +2719,43 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="24" x14ac:dyDescent="0.35">
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="15" t="s">
         <v>356</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="16" t="s">
         <v>360</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="16" t="s">
         <v>361</v>
       </c>
-      <c r="E19" s="18">
-        <v>1</v>
-      </c>
-      <c r="F19" s="18">
-        <v>1</v>
-      </c>
-      <c r="G19" s="18">
-        <v>1</v>
-      </c>
-      <c r="H19" s="18">
+      <c r="E19" s="16">
+        <v>1</v>
+      </c>
+      <c r="F19" s="16">
+        <v>1</v>
+      </c>
+      <c r="G19" s="16">
+        <v>1</v>
+      </c>
+      <c r="H19" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="24" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="17" t="s">
         <v>356</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="18" t="s">
         <v>362</v>
       </c>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="18" t="s">
         <v>363</v>
       </c>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20" t="e">
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
@@ -2676,25 +2764,25 @@
       <c r="A21" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="15" t="s">
         <v>364</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="16" t="s">
         <v>365</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="D21" s="16" t="s">
         <v>366</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="16">
         <v>691</v>
       </c>
-      <c r="F21" s="18">
+      <c r="F21" s="16">
         <v>972</v>
       </c>
-      <c r="G21" s="18">
+      <c r="G21" s="16">
         <v>493</v>
       </c>
-      <c r="H21" s="18">
+      <c r="H21" s="16">
         <f t="shared" si="0"/>
         <v>718.66666666666663</v>
       </c>
@@ -2703,107 +2791,107 @@
       <c r="A22" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="15" t="s">
         <v>367</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="16" t="s">
         <v>365</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="D22" s="16" t="s">
         <v>368</v>
       </c>
-      <c r="E22" s="18">
+      <c r="E22" s="16">
         <v>1E-3</v>
       </c>
-      <c r="F22" s="18">
+      <c r="F22" s="16">
         <v>1E-3</v>
       </c>
-      <c r="G22" s="18">
+      <c r="G22" s="16">
         <v>1E-3</v>
       </c>
-      <c r="H22" s="18">
+      <c r="H22" s="16">
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="15" t="s">
         <v>367</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="16" t="s">
         <v>369</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="D23" s="16" t="s">
         <v>370</v>
       </c>
-      <c r="E23" s="18">
-        <v>1</v>
-      </c>
-      <c r="F23" s="18">
-        <v>1</v>
-      </c>
-      <c r="G23" s="18">
-        <v>1</v>
-      </c>
-      <c r="H23" s="18">
+      <c r="E23" s="16">
+        <v>1</v>
+      </c>
+      <c r="F23" s="16">
+        <v>1</v>
+      </c>
+      <c r="G23" s="16">
+        <v>1</v>
+      </c>
+      <c r="H23" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="15" t="s">
         <v>367</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="16" t="s">
         <v>371</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="16" t="s">
         <v>372</v>
       </c>
-      <c r="E24" s="18">
+      <c r="E24" s="16">
         <v>9</v>
       </c>
-      <c r="F24" s="18">
+      <c r="F24" s="16">
         <v>9.3000000000000007</v>
       </c>
-      <c r="G24" s="18">
+      <c r="G24" s="16">
         <v>6.1</v>
       </c>
-      <c r="H24" s="18">
+      <c r="H24" s="16">
         <f t="shared" si="0"/>
         <v>8.1333333333333329</v>
       </c>
     </row>
     <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="17" t="s">
         <v>367</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="18" t="s">
         <v>369</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="D25" s="18" t="s">
         <v>373</v>
       </c>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="20"/>
-      <c r="H25" s="20" t="e">
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="19" t="s">
         <v>367</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="20" t="s">
         <v>374</v>
       </c>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="20" t="e">
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="18" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
@@ -2817,6 +2905,347 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="11" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
+      <c r="A1" s="49" t="s">
+        <v>267</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="K14" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:J14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2826,18 +3255,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
     </row>
     <row r="4" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -3056,433 +3485,433 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="18" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="13" t="s">
-        <v>425</v>
-      </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="B1" s="32" t="s">
+        <v>414</v>
+      </c>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
     </row>
     <row r="2" spans="2:8" ht="36" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="C2" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="15" t="s">
+      <c r="C2" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="13" t="s">
         <v>320</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="14" t="s">
         <v>321</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="F2" s="14" t="s">
         <v>322</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="14" t="s">
         <v>323</v>
       </c>
-      <c r="H2" s="16" t="s">
+      <c r="H2" s="14" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="15" t="s">
         <v>375</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="16" t="s">
         <v>336</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="16" t="s">
         <v>377</v>
       </c>
-      <c r="E3" s="18">
-        <v>1</v>
-      </c>
-      <c r="F3" s="18">
-        <v>1</v>
-      </c>
-      <c r="G3" s="18">
-        <v>1</v>
-      </c>
-      <c r="H3" s="18">
+      <c r="E3" s="16">
+        <v>1</v>
+      </c>
+      <c r="F3" s="16">
+        <v>1</v>
+      </c>
+      <c r="G3" s="16">
+        <v>1</v>
+      </c>
+      <c r="H3" s="16">
         <f t="shared" ref="H3:H30" si="0">AVERAGE(E3:G3)</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="15" t="s">
         <v>375</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="16" t="s">
         <v>338</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="16" t="s">
         <v>379</v>
       </c>
-      <c r="E4" s="18">
-        <v>1</v>
-      </c>
-      <c r="F4" s="18">
-        <v>1</v>
-      </c>
-      <c r="G4" s="18">
-        <v>1</v>
-      </c>
-      <c r="H4" s="18">
+      <c r="E4" s="16">
+        <v>1</v>
+      </c>
+      <c r="F4" s="16">
+        <v>1</v>
+      </c>
+      <c r="G4" s="16">
+        <v>1</v>
+      </c>
+      <c r="H4" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="15" t="s">
         <v>375</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="16" t="s">
         <v>340</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="16" t="s">
         <v>341</v>
       </c>
-      <c r="E5" s="18">
-        <v>1</v>
-      </c>
-      <c r="F5" s="18">
-        <v>1</v>
-      </c>
-      <c r="G5" s="18">
-        <v>1</v>
-      </c>
-      <c r="H5" s="18">
+      <c r="E5" s="16">
+        <v>1</v>
+      </c>
+      <c r="F5" s="16">
+        <v>1</v>
+      </c>
+      <c r="G5" s="16">
+        <v>1</v>
+      </c>
+      <c r="H5" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="15" t="s">
         <v>375</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="16" t="s">
         <v>378</v>
       </c>
-      <c r="E6" s="18">
-        <v>1</v>
-      </c>
-      <c r="F6" s="18">
-        <v>1</v>
-      </c>
-      <c r="G6" s="18">
-        <v>1</v>
-      </c>
-      <c r="H6" s="18">
+      <c r="E6" s="16">
+        <v>1</v>
+      </c>
+      <c r="F6" s="16">
+        <v>1</v>
+      </c>
+      <c r="G6" s="16">
+        <v>1</v>
+      </c>
+      <c r="H6" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="35.5" x14ac:dyDescent="0.35">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="15" t="s">
         <v>376</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="C7" s="24" t="s">
+        <v>391</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="E7" s="33" t="s">
         <v>403</v>
       </c>
-      <c r="D7" s="18" t="s">
-        <v>405</v>
-      </c>
-      <c r="E7" s="32" t="s">
-        <v>415</v>
-      </c>
-      <c r="F7" s="33"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="35"/>
     </row>
     <row r="8" spans="2:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="15" t="s">
         <v>376</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>404</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>406</v>
-      </c>
-      <c r="E8" s="35"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="37"/>
+      <c r="C8" s="16" t="s">
+        <v>392</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>394</v>
+      </c>
+      <c r="E8" s="36"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="38"/>
     </row>
     <row r="9" spans="2:8" ht="35.5" x14ac:dyDescent="0.35">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="15" t="s">
         <v>376</v>
       </c>
-      <c r="C9" s="18" t="s">
-        <v>407</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>408</v>
-      </c>
-      <c r="E9" s="35"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="37"/>
+      <c r="C9" s="16" t="s">
+        <v>395</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>396</v>
+      </c>
+      <c r="E9" s="36"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="38"/>
     </row>
     <row r="10" spans="2:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="15" t="s">
         <v>376</v>
       </c>
-      <c r="C10" s="18" t="s">
-        <v>409</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>410</v>
-      </c>
-      <c r="E10" s="35"/>
-      <c r="F10" s="36"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="37"/>
+      <c r="C10" s="16" t="s">
+        <v>397</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>398</v>
+      </c>
+      <c r="E10" s="36"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="38"/>
     </row>
     <row r="11" spans="2:8" ht="58.5" x14ac:dyDescent="0.35">
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="15" t="s">
         <v>376</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>411</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>412</v>
-      </c>
-      <c r="E11" s="35"/>
-      <c r="F11" s="36"/>
-      <c r="G11" s="36"/>
-      <c r="H11" s="37"/>
+      <c r="C11" s="16" t="s">
+        <v>399</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>400</v>
+      </c>
+      <c r="E11" s="36"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="38"/>
     </row>
     <row r="12" spans="2:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="15" t="s">
         <v>376</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>413</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>414</v>
-      </c>
-      <c r="E12" s="35"/>
-      <c r="F12" s="36"/>
-      <c r="G12" s="36"/>
-      <c r="H12" s="37"/>
+      <c r="C12" s="16" t="s">
+        <v>401</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>402</v>
+      </c>
+      <c r="E12" s="36"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="38"/>
     </row>
     <row r="13" spans="2:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="15" t="s">
         <v>376</v>
       </c>
-      <c r="C13" s="18" t="s">
-        <v>409</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>410</v>
-      </c>
-      <c r="E13" s="38"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="40"/>
+      <c r="C13" s="16" t="s">
+        <v>397</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>398</v>
+      </c>
+      <c r="E13" s="39"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="40"/>
+      <c r="H13" s="41"/>
     </row>
     <row r="14" spans="2:8" ht="24" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="17" t="s">
         <v>343</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="18" t="s">
         <v>344</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="D14" s="18" t="s">
         <v>345</v>
       </c>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20" t="e">
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B15" s="19"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
     </row>
     <row r="16" spans="2:8" ht="24" x14ac:dyDescent="0.35">
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="16" t="s">
         <v>347</v>
       </c>
-      <c r="E16" s="18">
-        <v>1</v>
-      </c>
-      <c r="F16" s="18">
-        <v>1</v>
-      </c>
-      <c r="G16" s="18">
-        <v>1</v>
-      </c>
-      <c r="H16" s="18">
+      <c r="E16" s="16">
+        <v>1</v>
+      </c>
+      <c r="F16" s="16">
+        <v>1</v>
+      </c>
+      <c r="G16" s="16">
+        <v>1</v>
+      </c>
+      <c r="H16" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="16" t="s">
         <v>348</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="16" t="s">
         <v>349</v>
       </c>
-      <c r="E17" s="18">
-        <v>1</v>
-      </c>
-      <c r="F17" s="18">
-        <v>1</v>
-      </c>
-      <c r="G17" s="18">
-        <v>1</v>
-      </c>
-      <c r="H17" s="18">
+      <c r="E17" s="16">
+        <v>1</v>
+      </c>
+      <c r="F17" s="16">
+        <v>1</v>
+      </c>
+      <c r="G17" s="16">
+        <v>1</v>
+      </c>
+      <c r="H17" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="16" t="s">
         <v>350</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="16" t="s">
         <v>351</v>
       </c>
-      <c r="E18" s="18">
-        <v>1</v>
-      </c>
-      <c r="F18" s="18">
-        <v>1</v>
-      </c>
-      <c r="G18" s="18">
-        <v>1</v>
-      </c>
-      <c r="H18" s="18">
+      <c r="E18" s="16">
+        <v>1</v>
+      </c>
+      <c r="F18" s="16">
+        <v>1</v>
+      </c>
+      <c r="G18" s="16">
+        <v>1</v>
+      </c>
+      <c r="H18" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="16" t="s">
         <v>352</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="16" t="s">
         <v>353</v>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="16">
         <v>5</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="16">
         <v>5</v>
       </c>
-      <c r="G19" s="18">
+      <c r="G19" s="16">
         <v>5</v>
       </c>
-      <c r="H19" s="18">
+      <c r="H19" s="16">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="16" t="s">
         <v>352</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="16" t="s">
         <v>354</v>
       </c>
-      <c r="E20" s="18">
+      <c r="E20" s="16">
         <v>5</v>
       </c>
-      <c r="F20" s="18">
+      <c r="F20" s="16">
         <v>5</v>
       </c>
-      <c r="G20" s="18">
+      <c r="G20" s="16">
         <v>5</v>
       </c>
-      <c r="H20" s="18">
+      <c r="H20" s="16">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="15" t="s">
         <v>343</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="16" t="s">
         <v>352</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="D21" s="16" t="s">
         <v>355</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="16">
         <v>5</v>
       </c>
-      <c r="F21" s="18">
+      <c r="F21" s="16">
         <v>5</v>
       </c>
-      <c r="G21" s="18">
+      <c r="G21" s="16">
         <v>5</v>
       </c>
-      <c r="H21" s="18">
+      <c r="H21" s="16">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="24" x14ac:dyDescent="0.35">
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="15" t="s">
         <v>356</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="16" t="s">
         <v>357</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="D22" s="16" t="s">
         <v>358</v>
       </c>
-      <c r="E22" s="18">
+      <c r="E22" s="16">
         <v>19.84</v>
       </c>
-      <c r="F22" s="18">
+      <c r="F22" s="16">
         <v>25.2</v>
       </c>
-      <c r="G22" s="18">
+      <c r="G22" s="16">
         <v>17.8</v>
       </c>
-      <c r="H22" s="18">
+      <c r="H22" s="16">
         <f t="shared" si="0"/>
         <v>20.946666666666669</v>
       </c>
@@ -3491,43 +3920,43 @@
       </c>
     </row>
     <row r="23" spans="1:9" ht="24" x14ac:dyDescent="0.35">
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="15" t="s">
         <v>356</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="16" t="s">
         <v>360</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="D23" s="16" t="s">
         <v>361</v>
       </c>
-      <c r="E23" s="18">
-        <v>1</v>
-      </c>
-      <c r="F23" s="18">
-        <v>1</v>
-      </c>
-      <c r="G23" s="18">
-        <v>1</v>
-      </c>
-      <c r="H23" s="18">
+      <c r="E23" s="16">
+        <v>1</v>
+      </c>
+      <c r="F23" s="16">
+        <v>1</v>
+      </c>
+      <c r="G23" s="16">
+        <v>1</v>
+      </c>
+      <c r="H23" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="24" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="17" t="s">
         <v>356</v>
       </c>
-      <c r="C24" s="20" t="s">
+      <c r="C24" s="18" t="s">
         <v>362</v>
       </c>
-      <c r="D24" s="20" t="s">
+      <c r="D24" s="18" t="s">
         <v>363</v>
       </c>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20" t="e">
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
@@ -3536,25 +3965,25 @@
       <c r="A25" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="15" t="s">
         <v>364</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="16" t="s">
         <v>365</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="D25" s="16" t="s">
         <v>366</v>
       </c>
-      <c r="E25" s="18">
+      <c r="E25" s="16">
         <v>2587</v>
       </c>
-      <c r="F25" s="18">
+      <c r="F25" s="16">
         <v>2654</v>
       </c>
-      <c r="G25" s="18">
+      <c r="G25" s="16">
         <v>2338</v>
       </c>
-      <c r="H25" s="18">
+      <c r="H25" s="16">
         <f t="shared" si="0"/>
         <v>2526.3333333333335</v>
       </c>
@@ -3563,107 +3992,107 @@
       <c r="A26" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="15" t="s">
         <v>367</v>
       </c>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="16" t="s">
         <v>365</v>
       </c>
-      <c r="D26" s="18" t="s">
+      <c r="D26" s="16" t="s">
         <v>368</v>
       </c>
-      <c r="E26" s="18">
+      <c r="E26" s="16">
         <v>2E-3</v>
       </c>
-      <c r="F26" s="18">
+      <c r="F26" s="16">
         <v>1E-3</v>
       </c>
-      <c r="G26" s="18">
+      <c r="G26" s="16">
         <v>2E-3</v>
       </c>
-      <c r="H26" s="18">
+      <c r="H26" s="16">
         <f t="shared" si="0"/>
         <v>1.6666666666666668E-3</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="15" t="s">
         <v>367</v>
       </c>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="16" t="s">
         <v>369</v>
       </c>
-      <c r="D27" s="18" t="s">
+      <c r="D27" s="16" t="s">
         <v>370</v>
       </c>
-      <c r="E27" s="18">
-        <v>1</v>
-      </c>
-      <c r="F27" s="18">
-        <v>1</v>
-      </c>
-      <c r="G27" s="18">
-        <v>1</v>
-      </c>
-      <c r="H27" s="18">
+      <c r="E27" s="16">
+        <v>1</v>
+      </c>
+      <c r="F27" s="16">
+        <v>1</v>
+      </c>
+      <c r="G27" s="16">
+        <v>1</v>
+      </c>
+      <c r="H27" s="16">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="15" t="s">
         <v>367</v>
       </c>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="16" t="s">
         <v>371</v>
       </c>
-      <c r="D28" s="18" t="s">
+      <c r="D28" s="16" t="s">
         <v>372</v>
       </c>
-      <c r="E28" s="18">
+      <c r="E28" s="16">
         <v>19</v>
       </c>
-      <c r="F28" s="18">
+      <c r="F28" s="16">
         <v>23</v>
       </c>
-      <c r="G28" s="18">
+      <c r="G28" s="16">
         <v>17</v>
       </c>
-      <c r="H28" s="18">
+      <c r="H28" s="16">
         <f t="shared" si="0"/>
         <v>19.666666666666668</v>
       </c>
     </row>
     <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="17" t="s">
         <v>367</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="18" t="s">
         <v>369</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="D29" s="18" t="s">
         <v>373</v>
       </c>
-      <c r="E29" s="20"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="20"/>
-      <c r="H29" s="20" t="e">
+      <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="18" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="19" t="s">
         <v>367</v>
       </c>
-      <c r="C30" s="22" t="s">
+      <c r="C30" s="20" t="s">
         <v>374</v>
       </c>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="20" t="e">
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="18" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
@@ -3678,11 +4107,624 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5475B8D2-64AB-42A9-918F-80E38A9F1FED}">
-  <dimension ref="C1:F12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA413DDE-FD08-44FA-9AE8-ADB21D1E6BEF}">
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="8.7265625" style="10"/>
+    <col min="1" max="1" width="8.7265625" style="11"/>
+    <col min="2" max="2" width="27" style="11" customWidth="1"/>
+    <col min="3" max="3" width="26" style="11" customWidth="1"/>
+    <col min="4" max="4" width="33.54296875" style="11" customWidth="1"/>
+    <col min="5" max="5" width="10" style="11" customWidth="1"/>
+    <col min="6" max="7" width="10.08984375" style="11" customWidth="1"/>
+    <col min="8" max="8" width="17.7265625" style="11" customWidth="1"/>
+    <col min="9" max="9" width="16.7265625" style="11" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8" ht="18" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B1" s="32" t="s">
+        <v>413</v>
+      </c>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+    </row>
+    <row r="2" spans="2:8" ht="36" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>320</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>321</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>322</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>323</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" ht="24" x14ac:dyDescent="0.35">
+      <c r="B3" s="15" t="s">
+        <v>375</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>336</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>377</v>
+      </c>
+      <c r="E3" s="16">
+        <v>1</v>
+      </c>
+      <c r="F3" s="16">
+        <v>1</v>
+      </c>
+      <c r="G3" s="16">
+        <v>1</v>
+      </c>
+      <c r="H3" s="16">
+        <f t="shared" ref="H3:H30" si="0">AVERAGE(E3:G3)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" ht="24" x14ac:dyDescent="0.35">
+      <c r="B4" s="15" t="s">
+        <v>375</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>338</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>379</v>
+      </c>
+      <c r="E4" s="16">
+        <v>1</v>
+      </c>
+      <c r="F4" s="16">
+        <v>1</v>
+      </c>
+      <c r="G4" s="16">
+        <v>1</v>
+      </c>
+      <c r="H4" s="16">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="24" x14ac:dyDescent="0.35">
+      <c r="B5" s="15" t="s">
+        <v>375</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>340</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>341</v>
+      </c>
+      <c r="E5" s="16">
+        <v>1</v>
+      </c>
+      <c r="F5" s="16">
+        <v>1</v>
+      </c>
+      <c r="G5" s="16">
+        <v>1</v>
+      </c>
+      <c r="H5" s="16">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" ht="24" x14ac:dyDescent="0.35">
+      <c r="B6" s="15" t="s">
+        <v>375</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>378</v>
+      </c>
+      <c r="E6" s="16">
+        <v>1</v>
+      </c>
+      <c r="F6" s="16">
+        <v>1</v>
+      </c>
+      <c r="G6" s="16">
+        <v>1</v>
+      </c>
+      <c r="H6" s="16">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" ht="35.5" x14ac:dyDescent="0.35">
+      <c r="B7" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>391</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="E7" s="33"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="35"/>
+    </row>
+    <row r="8" spans="2:8" ht="24" x14ac:dyDescent="0.35">
+      <c r="B8" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>392</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>394</v>
+      </c>
+      <c r="E8" s="36"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="38"/>
+    </row>
+    <row r="9" spans="2:8" ht="35.5" x14ac:dyDescent="0.35">
+      <c r="B9" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>395</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>396</v>
+      </c>
+      <c r="E9" s="36"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="38"/>
+    </row>
+    <row r="10" spans="2:8" ht="24" x14ac:dyDescent="0.35">
+      <c r="B10" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>397</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>398</v>
+      </c>
+      <c r="E10" s="36"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="38"/>
+    </row>
+    <row r="11" spans="2:8" ht="58.5" x14ac:dyDescent="0.35">
+      <c r="B11" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>399</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>400</v>
+      </c>
+      <c r="E11" s="36"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="38"/>
+    </row>
+    <row r="12" spans="2:8" ht="24" x14ac:dyDescent="0.35">
+      <c r="B12" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>401</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>402</v>
+      </c>
+      <c r="E12" s="36"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="38"/>
+    </row>
+    <row r="13" spans="2:8" ht="24" x14ac:dyDescent="0.35">
+      <c r="B13" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>397</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>398</v>
+      </c>
+      <c r="E13" s="39"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="40"/>
+      <c r="H13" s="41"/>
+    </row>
+    <row r="14" spans="2:8" ht="24" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="17" t="s">
+        <v>343</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>344</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B15" s="17"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+    </row>
+    <row r="16" spans="2:8" ht="24" x14ac:dyDescent="0.35">
+      <c r="B16" s="15" t="s">
+        <v>343</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>346</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>347</v>
+      </c>
+      <c r="E16" s="16">
+        <v>1</v>
+      </c>
+      <c r="F16" s="16">
+        <v>1</v>
+      </c>
+      <c r="G16" s="16">
+        <v>1</v>
+      </c>
+      <c r="H16" s="16">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B17" s="15" t="s">
+        <v>343</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>348</v>
+      </c>
+      <c r="D17" s="16" t="s">
+        <v>349</v>
+      </c>
+      <c r="E17" s="16">
+        <v>1</v>
+      </c>
+      <c r="F17" s="16">
+        <v>1</v>
+      </c>
+      <c r="G17" s="16">
+        <v>1</v>
+      </c>
+      <c r="H17" s="16">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B18" s="15" t="s">
+        <v>343</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>350</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>351</v>
+      </c>
+      <c r="E18" s="16">
+        <v>1</v>
+      </c>
+      <c r="F18" s="16">
+        <v>1</v>
+      </c>
+      <c r="G18" s="16">
+        <v>1</v>
+      </c>
+      <c r="H18" s="16">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B19" s="15" t="s">
+        <v>343</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="D19" s="16" t="s">
+        <v>353</v>
+      </c>
+      <c r="E19" s="16">
+        <v>5</v>
+      </c>
+      <c r="F19" s="16">
+        <v>5</v>
+      </c>
+      <c r="G19" s="16">
+        <v>5</v>
+      </c>
+      <c r="H19" s="16">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B20" s="15" t="s">
+        <v>343</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>354</v>
+      </c>
+      <c r="E20" s="16">
+        <v>5</v>
+      </c>
+      <c r="F20" s="16">
+        <v>5</v>
+      </c>
+      <c r="G20" s="16">
+        <v>5</v>
+      </c>
+      <c r="H20" s="16">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B21" s="15" t="s">
+        <v>343</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>355</v>
+      </c>
+      <c r="E21" s="16">
+        <v>5</v>
+      </c>
+      <c r="F21" s="16">
+        <v>5</v>
+      </c>
+      <c r="G21" s="16">
+        <v>5</v>
+      </c>
+      <c r="H21" s="16">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="24" x14ac:dyDescent="0.35">
+      <c r="B22" s="15" t="s">
+        <v>356</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>357</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="E22" s="16">
+        <v>17.8</v>
+      </c>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16">
+        <f t="shared" si="0"/>
+        <v>17.8</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="24" x14ac:dyDescent="0.35">
+      <c r="B23" s="15" t="s">
+        <v>356</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>360</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="E23" s="16">
+        <v>1</v>
+      </c>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="16">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="24" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="17" t="s">
+        <v>356</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>363</v>
+      </c>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="24" x14ac:dyDescent="0.35">
+      <c r="A25" s="11" t="s">
+        <v>325</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>364</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>366</v>
+      </c>
+      <c r="E25" s="16">
+        <v>45517</v>
+      </c>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="16">
+        <f t="shared" si="0"/>
+        <v>45517</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="11" t="s">
+        <v>325</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>367</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="E26" s="16">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="16">
+        <f t="shared" si="0"/>
+        <v>4.9000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B27" s="15" t="s">
+        <v>367</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>370</v>
+      </c>
+      <c r="E27" s="16">
+        <v>1</v>
+      </c>
+      <c r="F27" s="16"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="16">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B28" s="15" t="s">
+        <v>367</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>371</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>372</v>
+      </c>
+      <c r="E28" s="16">
+        <v>352</v>
+      </c>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16">
+        <f t="shared" si="0"/>
+        <v>352</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="17" t="s">
+        <v>367</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>369</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>373</v>
+      </c>
+      <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="18" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B30" s="19" t="s">
+        <v>367</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>374</v>
+      </c>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="18" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="E7:H13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5475B8D2-64AB-42A9-918F-80E38A9F1FED}">
+  <dimension ref="B1:F13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.7265625" style="10"/>
+    <col min="2" max="2" width="10.26953125" style="31" customWidth="1"/>
     <col min="3" max="3" width="21.26953125" style="10" customWidth="1"/>
     <col min="4" max="4" width="32.08984375" style="10" customWidth="1"/>
     <col min="5" max="5" width="38.81640625" style="10" customWidth="1"/>
@@ -3690,128 +4732,163 @@
     <col min="7" max="16384" width="8.7265625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C1" s="27" t="s">
-        <v>402</v>
-      </c>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-    </row>
-    <row r="2" spans="3:6" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="C2" s="28" t="s">
+    <row r="1" spans="2:6" ht="16" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="27"/>
+      <c r="C1" s="42" t="s">
+        <v>390</v>
+      </c>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="43"/>
+    </row>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B2" s="28" t="s">
+        <v>416</v>
+      </c>
+      <c r="C2" s="25" t="s">
         <v>380</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="25" t="s">
         <v>381</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="E2" s="25" t="s">
         <v>382</v>
       </c>
-      <c r="F2" s="30" t="s">
+      <c r="F2" s="26" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="3" spans="3:6" ht="58.5" x14ac:dyDescent="0.35">
-      <c r="C3" s="17" t="s">
+    <row r="3" spans="2:6" ht="24" x14ac:dyDescent="0.35">
+      <c r="B3" s="29">
+        <v>1</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>415</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>417</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>424</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="58.5" x14ac:dyDescent="0.35">
+      <c r="B4" s="29">
+        <v>2</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>422</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>421</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>420</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="47" x14ac:dyDescent="0.35">
+      <c r="B5" s="29">
+        <v>3</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>419</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>423</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" s="11" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="44"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="46"/>
+    </row>
+    <row r="7" spans="2:6" ht="24" x14ac:dyDescent="0.35">
+      <c r="B7" s="29"/>
+      <c r="C7" s="16" t="s">
+        <v>426</v>
+      </c>
+      <c r="D7" s="16" t="s">
         <v>384</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="E7" s="16" t="s">
+        <v>429</v>
+      </c>
+      <c r="F7" s="21" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="24" x14ac:dyDescent="0.35">
+      <c r="B8" s="29"/>
+      <c r="C8" s="16" t="s">
+        <v>427</v>
+      </c>
+      <c r="D8" s="16" t="s">
         <v>385</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E8" s="16"/>
+      <c r="F8" s="21"/>
+    </row>
+    <row r="9" spans="2:6" ht="24" x14ac:dyDescent="0.35">
+      <c r="B9" s="29"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16" t="s">
         <v>386</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="E9" s="16"/>
+      <c r="F9" s="21"/>
+    </row>
+    <row r="10" spans="2:6" ht="24" x14ac:dyDescent="0.35">
+      <c r="B10" s="29"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="4" spans="3:6" ht="58.5" x14ac:dyDescent="0.35">
-      <c r="C4" s="17" t="s">
+      <c r="E10" s="16"/>
+      <c r="F10" s="21"/>
+    </row>
+    <row r="11" spans="2:6" ht="24" x14ac:dyDescent="0.35">
+      <c r="B11" s="29"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16" t="s">
         <v>388</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="E11" s="16"/>
+      <c r="F11" s="21"/>
+    </row>
+    <row r="12" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="30"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22" t="s">
         <v>389</v>
       </c>
-      <c r="E4" s="18" t="s">
-        <v>390</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="5" spans="3:6" ht="47" x14ac:dyDescent="0.35">
-      <c r="C5" s="17" t="s">
-        <v>392</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>393</v>
-      </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="23"/>
-    </row>
-    <row r="6" spans="3:6" ht="24" x14ac:dyDescent="0.35">
-      <c r="C6" s="17" t="s">
-        <v>394</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>395</v>
-      </c>
-      <c r="E6" s="18"/>
-      <c r="F6" s="23" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="7" spans="3:6" ht="24" x14ac:dyDescent="0.35">
-      <c r="C7" s="17"/>
-      <c r="D7" s="18" t="s">
-        <v>397</v>
-      </c>
-      <c r="E7" s="18"/>
-      <c r="F7" s="23"/>
-    </row>
-    <row r="8" spans="3:6" ht="24" x14ac:dyDescent="0.35">
-      <c r="C8" s="17"/>
-      <c r="D8" s="18" t="s">
-        <v>398</v>
-      </c>
-      <c r="E8" s="18"/>
-      <c r="F8" s="23"/>
-    </row>
-    <row r="9" spans="3:6" ht="24" x14ac:dyDescent="0.35">
-      <c r="C9" s="17"/>
-      <c r="D9" s="18" t="s">
-        <v>399</v>
-      </c>
-      <c r="E9" s="18"/>
-      <c r="F9" s="23"/>
-    </row>
-    <row r="10" spans="3:6" ht="24" x14ac:dyDescent="0.35">
-      <c r="C10" s="17"/>
-      <c r="D10" s="18" t="s">
-        <v>400</v>
-      </c>
-      <c r="E10" s="18"/>
-      <c r="F10" s="23"/>
-    </row>
-    <row r="11" spans="3:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C11" s="24"/>
-      <c r="D11" s="25" t="s">
-        <v>401</v>
-      </c>
-      <c r="E11" s="25"/>
-      <c r="F11" s="26"/>
-    </row>
-    <row r="12" spans="3:6" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="23"/>
+    </row>
+    <row r="13" spans="2:6" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="C1:F1"/>
+    <mergeCell ref="B6:F6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3821,32 +4898,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="41" t="s">
-        <v>416</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
+      <c r="A1" s="48" t="s">
+        <v>404</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -4307,7 +5384,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4317,19 +5394,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="41" t="s">
-        <v>417</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
+      <c r="A1" s="48" t="s">
+        <v>405</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -4900,7 +5977,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4910,19 +5987,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="49" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -4974,7 +6051,7 @@
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
-        <v>418</v>
+        <v>406</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>15</v>
@@ -5051,7 +6128,7 @@
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3" t="s">
-        <v>419</v>
+        <v>407</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>15</v>
@@ -5159,7 +6236,7 @@
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3" t="s">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>15</v>
@@ -5186,7 +6263,7 @@
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3" t="s">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>15</v>
@@ -5213,7 +6290,7 @@
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3" t="s">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>15</v>
@@ -5240,7 +6317,7 @@
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3" t="s">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>15</v>
@@ -5267,7 +6344,7 @@
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3" t="s">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>15</v>
@@ -5416,7 +6493,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -5426,19 +6503,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="41" t="s">
-        <v>421</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
+      <c r="A1" s="48" t="s">
+        <v>409</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -6077,7 +7154,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -6087,19 +7164,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="41" t="s">
-        <v>422</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
+      <c r="A1" s="48" t="s">
+        <v>410</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -6625,347 +7702,6 @@
       <c r="G30" s="9" t="s">
         <v>16</v>
       </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="11" width="15" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="12" t="s">
-        <v>267</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3" t="s">
-        <v>423</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="K6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3" t="s">
-        <v>424</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="K14" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>